<commit_message>
Sync planning SharePoint : S43
</commit_message>
<xml_diff>
--- a/Plannings 2026 S43.xlsx
+++ b/Plannings 2026 S43.xlsx
@@ -7899,13 +7899,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB575D56-E356-42B5-9EFF-E3D5DD1ABCE5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D0D1C95-5228-4624-9B76-43ECD3B7BD5A}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65FCA938-E5F7-4190-BE81-45E032BF79CB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CDB295C-FAF5-4737-A65B-819F0DFAEBCE}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E8CE58B-3F9B-4BB1-8E4C-BB6136340EED}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE64BB12-E752-4756-92B1-EDBE0BCAFCF4}"/>
 </file>
</xml_diff>